<commit_message>
Days 31 to 60 plus October news posts: slides, LinkedIn PDFs, captions, schedule, film scripts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TW9n8unhL8LSAM1TzockVG
</commit_message>
<xml_diff>
--- a/plan90.xlsx
+++ b/plan90.xlsx
@@ -2237,12 +2237,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>What Just Happened 01</t>
+          <t>What Changed 01</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>This just changed for every coach selling online. Let me explain.</t>
+          <t>Last month, the CBN asked a question about “pay small small”.</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>News, picked 2 days before</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Your family calls it “that your online thing”. Fix that in one sentence.</t>
+          <t>Your family calls it “that your online thing”.</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2732,12 +2732,12 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>This Week in 60 Seconds</t>
+          <t>News in 60 Seconds</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>3 things that happened this week that your competitors missed.</t>
+          <t>3 things your competitors missed.</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>News, picked 2 days before</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2807,7 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>You film, I script (designed fallback)</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Your spouse thinks online business is “yahoo”. Don't argue. Do this.</t>
+          <t>Your spouse thinks your online business is “yahoo”.</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -3502,12 +3502,12 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>This Week in 60 Seconds</t>
+          <t>News in 60 Seconds</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>3 things that happened this week that your competitors missed.</t>
+          <t>3 things to know before the holiday rush.</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr"/>
@@ -3518,7 +3518,7 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>News, picked 2 days before</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -3888,7 +3888,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Your partner is your first customer service test.</t>
+          <t>Your partner is your first clarity test.</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -4268,12 +4268,12 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>This Week in 60 Seconds</t>
+          <t>News in 60 Seconds</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>3 things that happened this week that your competitors missed.</t>
+          <t>3 changes your competitors missed.</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr"/>
@@ -4284,7 +4284,7 @@
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>News, picked 2 days before</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>The mistake that cost me a client, and what I do now.</t>
+          <t>I lost a $500 job because of one word.</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>You film, I script (designed fallback)</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Black Friday: discount or bonus? Do the math before you slash your price.</t>
+          <t>Discount or bonus? Do the math before you slash your price.</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
@@ -4539,12 +4539,12 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>What Just Happened</t>
+          <t>What Changed</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>This just changed for every coach selling online. Let me explain.</t>
+          <t>WhatsApp started charging businesses for replies.</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr"/>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>News, picked 2 days before</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -4595,7 +4595,7 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Steal this: the Black Friday waitlist message.</t>
+          <t>The Black Friday waitlist message.</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -4650,7 +4650,7 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Friends who don't support your business: stop doing these 3 things.</t>
+          <t>Friends not supporting your business? Stop doing these 3 things.</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -4925,7 +4925,7 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Working with your spouse? 4 rules before you destroy your marriage.</t>
+          <t>4 rules before you destroy your marriage.</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>The coach who follows up wins. Not the coach who's best.</t>
+          <t>The business that follows up wins. Not the one that's best.</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
@@ -5030,12 +5030,12 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>This Week in 60 Seconds</t>
+          <t>News in 60 Seconds</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>3 things that happened this week that your competitors missed.</t>
+          <t>3 numbers that should change your Black Friday prices.</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr"/>
@@ -5046,7 +5046,7 @@
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>News, picked 2 days before</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -5086,7 +5086,7 @@
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Things I will never do for a client, even for money.</t>
+          <t>Things I will never do for a client.</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
-          <t>You film, I script (designed fallback)</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -5251,7 +5251,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Autopsy 3: a Black Friday offer post.</t>
+          <t>I found 4 leaks in this Black Friday post.</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
@@ -5301,12 +5301,12 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>What Just Happened</t>
+          <t>What Changed</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>This just changed for every coach selling online. Let me explain.</t>
+          <t>For some Facebook Pages, link posts are becoming a paid feature.</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr"/>
@@ -5317,7 +5317,7 @@
       </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
-          <t>News, picked 2 days before</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -5522,7 +5522,7 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>What 3 working days of a Leak Map looks like.</t>
+          <t>What 3 working days of a Leak Map look like.</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
@@ -5577,7 +5577,7 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Today is the last day to book a Black Friday Leak Map.</t>
+          <t>Last day to book a Black Friday Leak Map.</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
@@ -5792,12 +5792,12 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>This Week in 60 Seconds</t>
+          <t>News in 60 Seconds</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>3 things that happened this week that your competitors missed.</t>
+          <t>3 signals of where selling online is going next.</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr"/>
@@ -5808,7 +5808,7 @@
       </c>
       <c r="K98" s="2" t="inlineStr">
         <is>
-          <t>News, picked 2 days before</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -5848,7 +5848,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>A day of writing a sales page in Lagos.</t>
+          <t>How a sales page gets made in Lagos.</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
@@ -5863,7 +5863,7 @@
       </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
-          <t>You film, I script (designed fallback)</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -6063,12 +6063,12 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>What Just Happened</t>
+          <t>What Changed</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>This just changed for every coach selling online. Let me explain.</t>
+          <t>Jumia says Nigeria orders rose 34%.</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr"/>
@@ -6079,7 +6079,7 @@
       </c>
       <c r="K103" s="2" t="inlineStr">
         <is>
-          <t>News, picked 2 days before</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -6229,7 +6229,7 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>“I'm still building my audience” is how coaches hide from selling.</t>
+          <t>“I'm still building my audience” is how businesses hide from selling.</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
@@ -6554,12 +6554,12 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>This Week in 60 Seconds</t>
+          <t>News in 60 Seconds</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>3 things that happened this week that your competitors missed.</t>
+          <t>3 things from the news to check this week.</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr"/>
@@ -6570,7 +6570,7 @@
       </c>
       <c r="K112" s="2" t="inlineStr">
         <is>
-          <t>News, picked 2 days before</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -6610,7 +6610,7 @@
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>What I would tell myself on day 1 of copywriting.</t>
+          <t>What I'd tell myself on day 1 of copywriting.</t>
         </is>
       </c>
       <c r="I113" s="2" t="inlineStr">
@@ -6625,7 +6625,7 @@
       </c>
       <c r="K113" s="2" t="inlineStr">
         <is>
-          <t>You film, I script (designed fallback)</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -6665,7 +6665,7 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>This week somebody less talented than you will make more money. Here's why.</t>
+          <t>This week, someone less talented than you will make more money. Here's why.</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
@@ -6720,7 +6720,7 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>Black Friday week: the 4 posts to make, and when.</t>
+          <t>The 4 posts to make, and when.</t>
         </is>
       </c>
       <c r="I115" s="2" t="inlineStr">
@@ -6825,12 +6825,12 @@
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>What Just Happened</t>
+          <t>What Changed</t>
         </is>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>This just changed for every coach selling online. Let me explain.</t>
+          <t>The Lagos tax agency is testing a 5% withholding tax on creator payouts.</t>
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr"/>
@@ -6841,7 +6841,7 @@
       </c>
       <c r="K117" s="2" t="inlineStr">
         <is>
-          <t>News, picked 2 days before</t>
+          <t>New, needs your approval</t>
         </is>
       </c>
     </row>
@@ -6881,7 +6881,7 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>Steal this: the message for people who clicked but didn't pay.</t>
+          <t>The message for people who clicked but didn't pay.</t>
         </is>
       </c>
       <c r="I118" s="2" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Tomorrow is Black Friday. Fix this one leak tonight.</t>
+          <t>Fix this one leak tonight.</t>
         </is>
       </c>
       <c r="I121" s="2" t="inlineStr">
@@ -7316,7 +7316,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>This Week in 60 Seconds</t>
+          <t>News in 60 Seconds</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>What Just Happened</t>
+          <t>What Changed</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>This Week in 60 Seconds</t>
+          <t>News in 60 Seconds</t>
         </is>
       </c>
       <c r="H140" s="2" t="inlineStr">
@@ -8349,7 +8349,7 @@
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>What Just Happened</t>
+          <t>What Changed</t>
         </is>
       </c>
       <c r="H145" s="2" t="inlineStr">
@@ -8840,7 +8840,7 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>This Week in 60 Seconds</t>
+          <t>News in 60 Seconds</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
@@ -9111,7 +9111,7 @@
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>What Just Happened</t>
+          <t>What Changed</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr">
@@ -9602,7 +9602,7 @@
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>This Week in 60 Seconds</t>
+          <t>News in 60 Seconds</t>
         </is>
       </c>
       <c r="H168" s="2" t="inlineStr">
@@ -9873,7 +9873,7 @@
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>What Just Happened</t>
+          <t>What Changed</t>
         </is>
       </c>
       <c r="H173" s="2" t="inlineStr">

</xml_diff>